<commit_message>
Annotated M Uchmanowicz extractions with PMIDs. Retrieved additional paywalled full-text PDFs.
</commit_message>
<xml_diff>
--- a/lit_review_manual/m_uchmanowicz_goldStandard_list.xlsx
+++ b/lit_review_manual/m_uchmanowicz_goldStandard_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{588FCF7B-1517-4033-B766-2BC241E73B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF5EE6E-AB8B-4ECB-878A-8D4732DD15D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="320">
   <si>
     <t xml:space="preserve">uniprot accession </t>
   </si>
@@ -991,6 +991,12 @@
   </si>
   <si>
     <t>Human homologue</t>
+  </si>
+  <si>
+    <t>PMID</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -2752,7 +2758,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99CD300C-8547-427F-A062-58196212E640}">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -2761,7 +2767,7 @@
     <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>213</v>
       </c>
@@ -2777,8 +2783,11 @@
       <c r="E1" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -2791,11 +2800,14 @@
       <c r="D2" t="s">
         <v>216</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="4" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2">
+        <v>39208803</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -2811,8 +2823,11 @@
       <c r="E3" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3">
+        <v>39208803</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -2828,32 +2843,71 @@
       <c r="E4" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4">
+        <v>32499527</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>319</v>
+      </c>
+      <c r="B5" t="s">
+        <v>319</v>
+      </c>
+      <c r="C5" t="s">
+        <v>319</v>
+      </c>
       <c r="D5" t="s">
         <v>222</v>
       </c>
       <c r="E5" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5">
+        <v>32499527</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>319</v>
+      </c>
+      <c r="B6" t="s">
+        <v>319</v>
+      </c>
+      <c r="C6" t="s">
+        <v>319</v>
+      </c>
       <c r="D6" t="s">
         <v>223</v>
       </c>
       <c r="E6" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F6">
+        <v>32499527</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>319</v>
+      </c>
+      <c r="B7" t="s">
+        <v>319</v>
+      </c>
+      <c r="C7" t="s">
+        <v>319</v>
+      </c>
       <c r="D7" t="s">
         <v>224</v>
       </c>
       <c r="E7" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F7">
+        <v>32499527</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -2869,24 +2923,51 @@
       <c r="E8" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F8">
+        <v>32499527</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>319</v>
+      </c>
+      <c r="B9" t="s">
+        <v>319</v>
+      </c>
+      <c r="C9" t="s">
+        <v>319</v>
+      </c>
       <c r="D9" t="s">
         <v>227</v>
       </c>
       <c r="E9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F9">
+        <v>32499527</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>319</v>
+      </c>
+      <c r="B10" t="s">
+        <v>319</v>
+      </c>
+      <c r="C10" t="s">
+        <v>319</v>
+      </c>
       <c r="D10" t="s">
         <v>228</v>
       </c>
       <c r="E10" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F10">
+        <v>32499527</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>86</v>
       </c>
@@ -2902,8 +2983,11 @@
       <c r="E11" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F11">
+        <v>39208803</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -2919,8 +3003,11 @@
       <c r="E12" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F12">
+        <v>36302390</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>77</v>
       </c>
@@ -2936,8 +3023,11 @@
       <c r="E13" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F13">
+        <v>36302390</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -2953,32 +3043,71 @@
       <c r="E14" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F14">
+        <v>36302390</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>319</v>
+      </c>
+      <c r="B15" t="s">
+        <v>319</v>
+      </c>
+      <c r="C15" t="s">
+        <v>319</v>
+      </c>
       <c r="D15" t="s">
         <v>242</v>
       </c>
       <c r="E15" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F15">
+        <v>36302390</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>319</v>
+      </c>
+      <c r="B16" t="s">
+        <v>319</v>
+      </c>
+      <c r="C16" t="s">
+        <v>319</v>
+      </c>
       <c r="D16" t="s">
         <v>243</v>
       </c>
       <c r="E16" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F16">
+        <v>36302390</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>319</v>
+      </c>
+      <c r="B17" t="s">
+        <v>319</v>
+      </c>
+      <c r="C17" t="s">
+        <v>319</v>
+      </c>
       <c r="D17" t="s">
         <v>244</v>
       </c>
       <c r="E17" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F17">
+        <v>36302390</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>81</v>
       </c>
@@ -2994,8 +3123,11 @@
       <c r="E18" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F18">
+        <v>36302390</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>164</v>
       </c>
@@ -3011,8 +3143,17 @@
       <c r="E19" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F19">
+        <v>38509367</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>319</v>
+      </c>
+      <c r="B20" t="s">
+        <v>319</v>
+      </c>
       <c r="C20" t="s">
         <v>251</v>
       </c>
@@ -3022,8 +3163,11 @@
       <c r="E20" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F20">
+        <v>29549035</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>254</v>
       </c>
@@ -3039,8 +3183,11 @@
       <c r="E21" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F21">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>259</v>
       </c>
@@ -3056,8 +3203,11 @@
       <c r="E22" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F22">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>263</v>
       </c>
@@ -3073,8 +3223,11 @@
       <c r="E23" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F23">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>267</v>
       </c>
@@ -3090,8 +3243,11 @@
       <c r="E24" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F24">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>271</v>
       </c>
@@ -3107,8 +3263,11 @@
       <c r="E25" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F25">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>275</v>
       </c>
@@ -3124,8 +3283,11 @@
       <c r="E26" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F26">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>279</v>
       </c>
@@ -3141,8 +3303,11 @@
       <c r="E27" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F27">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>283</v>
       </c>
@@ -3158,8 +3323,11 @@
       <c r="E28" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F28">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>287</v>
       </c>
@@ -3175,8 +3343,11 @@
       <c r="E29" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F29">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>291</v>
       </c>
@@ -3192,8 +3363,11 @@
       <c r="E30" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F30">
+        <v>32937646</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>295</v>
       </c>
@@ -3209,8 +3383,11 @@
       <c r="E31" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F31">
+        <v>32877915</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>300</v>
       </c>
@@ -3226,8 +3403,11 @@
       <c r="E32" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F32">
+        <v>32877915</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>303</v>
       </c>
@@ -3243,8 +3423,11 @@
       <c r="E33" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F33">
+        <v>39083849</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>307</v>
       </c>
@@ -3260,8 +3443,11 @@
       <c r="E34" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F34">
+        <v>25131990</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>311</v>
       </c>
@@ -3276,6 +3462,9 @@
       </c>
       <c r="E35" t="s">
         <v>315</v>
+      </c>
+      <c r="F35">
+        <v>31019074</v>
       </c>
     </row>
   </sheetData>
@@ -3302,6 +3491,7 @@
     <hyperlink ref="E33" r:id="rId20" xr:uid="{31B2A8C7-7B19-4E7D-ADF7-C8FC81DD7402}"/>
     <hyperlink ref="E35" r:id="rId21" xr:uid="{3E3EE966-6694-4A85-802E-E4C9C4C738F2}"/>
     <hyperlink ref="E34" r:id="rId22" xr:uid="{0A81A9AA-442D-472B-8246-E340B5D51842}"/>
+    <hyperlink ref="E2" r:id="rId23" xr:uid="{A9CA86A1-BFA9-4737-BDAC-CCFB9B547CF2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>